<commit_message>
README with measured results, artwork and a sharper demo video
- README following the project style: hero, measured metrics strip, real showcase, how it works, what's inside, use, eval results, architecture, decisions, development
- web/scripts/readme-assets.mjs generates the artwork in docs/readme (light and dark) and composes the showcase from the English review screen the demo captures
- The demo is now recorded from Chromium's screencast at 1920x1200 and encoded to MP4 by a pinned ffmpeg image, with a poster; screenshots at the same scale
</commit_message>
<xml_diff>
--- a/docs/demo/facturas-ejemplo.xlsx
+++ b/docs/demo/facturas-ejemplo.xlsx
@@ -56,7 +56,7 @@
     <x:t>Total</x:t>
   </x:si>
   <x:si>
-    <x:t>01a163c1-f362-762f-973b-a2ae6ea5958a</x:t>
+    <x:t>01a163cf-f6c6-73b3-a4fb-6c4b44aee663</x:t>
   </x:si>
   <x:si>
     <x:t>sample-09.pdf</x:t>
@@ -83,7 +83,7 @@
     <x:t>USD</x:t>
   </x:si>
   <x:si>
-    <x:t>01a163c1-f36a-7c24-a7a8-6663d2a7b6d2</x:t>
+    <x:t>01a163cf-f6c9-7edf-8d6c-420eecec9bd7</x:t>
   </x:si>
   <x:si>
     <x:t>sample-10.png</x:t>
@@ -101,7 +101,7 @@
     <x:t>INV-001270</x:t>
   </x:si>
   <x:si>
-    <x:t>01a163c1-f36b-7f81-a779-f53affad2516</x:t>
+    <x:t>01a163cf-f6cb-7d7c-9d11-35f5d6fc6af2</x:t>
   </x:si>
   <x:si>
     <x:t>sample-11.jpg</x:t>

</xml_diff>

<commit_message>
Demo re-recorded with the built-in examples and localized rule details
The batch is built with the example buttons, the country follows the first one, and the review scene points at the rule's numbers in Spanish (taken from the reading, not hard-coded). README showcase regenerated from the new English review screen; its alt text no longer claims an uncertain field this run did not have.
</commit_message>
<xml_diff>
--- a/docs/demo/facturas-ejemplo.xlsx
+++ b/docs/demo/facturas-ejemplo.xlsx
@@ -56,7 +56,7 @@
     <x:t>Total</x:t>
   </x:si>
   <x:si>
-    <x:t>01a163cf-f6c6-73b3-a4fb-6c4b44aee663</x:t>
+    <x:t>01a16458-2238-71a7-b384-681fb17fc030</x:t>
   </x:si>
   <x:si>
     <x:t>sample-09.pdf</x:t>
@@ -83,7 +83,7 @@
     <x:t>USD</x:t>
   </x:si>
   <x:si>
-    <x:t>01a163cf-f6c9-7edf-8d6c-420eecec9bd7</x:t>
+    <x:t>01a16458-223e-7fcc-ae14-795888396781</x:t>
   </x:si>
   <x:si>
     <x:t>sample-10.png</x:t>
@@ -101,7 +101,7 @@
     <x:t>INV-001270</x:t>
   </x:si>
   <x:si>
-    <x:t>01a163cf-f6cb-7d7c-9d11-35f5d6fc6af2</x:t>
+    <x:t>01a16458-2240-7d74-b4cb-36170ec1aa4b</x:t>
   </x:si>
   <x:si>
     <x:t>sample-11.jpg</x:t>

</xml_diff>